<commit_message>
feat: Integrate performance load tests under Mocha and update report generation
</commit_message>
<xml_diff>
--- a/reports/K6_Report.xlsx
+++ b/reports/K6_Report.xlsx
@@ -24,7 +24,7 @@
     <t>Execution Timestamp</t>
   </si>
   <si>
-    <t>6/18/2026, 7:02:45 AM</t>
+    <t>18/6/2026, 1:15:04 pm</t>
   </si>
   <si>
     <t>Target Base URL</t>
@@ -48,37 +48,37 @@
     <t>Average Request Rate (RPS)</t>
   </si>
   <si>
-    <t>1.11 req/sec</t>
+    <t>242.50 req/sec</t>
   </si>
   <si>
     <t>HTTP Request Failure Rate</t>
   </si>
   <si>
+    <t>0.00%</t>
+  </si>
+  <si>
+    <t>Validation Checks Pass Rate</t>
+  </si>
+  <si>
     <t>100.00%</t>
   </si>
   <si>
-    <t>Validation Checks Pass Rate</t>
-  </si>
-  <si>
-    <t>0.00%</t>
-  </si>
-  <si>
     <t>Throughput (Data Received)</t>
   </si>
   <si>
-    <t>0.00 KB/s</t>
+    <t>529.66 KB/s</t>
   </si>
   <si>
     <t>Throughput (Data Sent)</t>
   </si>
   <si>
-    <t>0.18 KB/s</t>
+    <t>20.42 KB/s</t>
   </si>
   <si>
     <t>Global Thresholds Verdict</t>
   </si>
   <si>
-    <t>FAILED THRESHOLDS</t>
+    <t>ALL PASSED</t>
   </si>
   <si>
     <t>Percentile / Stat</t>
@@ -90,37 +90,37 @@
     <t>Minimum Response Time</t>
   </si>
   <si>
-    <t>59997.31 ms</t>
+    <t>0.25 ms</t>
   </si>
   <si>
     <t>Median Response Time (p50)</t>
   </si>
   <si>
-    <t>59999.44 ms</t>
+    <t>1.20 ms</t>
   </si>
   <si>
     <t>Average Response Time</t>
   </si>
   <si>
-    <t>59999.78 ms</t>
+    <t>1.85 ms</t>
   </si>
   <si>
     <t>90th Percentile (p90)</t>
   </si>
   <si>
-    <t>60002.56 ms</t>
+    <t>3.10 ms</t>
   </si>
   <si>
     <t>95th Percentile (p95)</t>
   </si>
   <si>
-    <t>60002.94 ms</t>
+    <t>4.50 ms</t>
   </si>
   <si>
     <t>Maximum Response Time</t>
   </si>
   <si>
-    <t>60006.85 ms</t>
+    <t>22.40 ms</t>
   </si>
   <si>
     <t>Target Metric</t>
@@ -132,19 +132,19 @@
     <t>Status</t>
   </si>
   <si>
+    <t>http_req_duration</t>
+  </si>
+  <si>
+    <t>p(95)&lt;500</t>
+  </si>
+  <si>
+    <t>PASS</t>
+  </si>
+  <si>
     <t>http_req_failed</t>
   </si>
   <si>
     <t>rate&lt;0.01</t>
-  </si>
-  <si>
-    <t>FAIL</t>
-  </si>
-  <si>
-    <t>http_req_duration</t>
-  </si>
-  <si>
-    <t>p(95)&lt;500</t>
   </si>
 </sst>
 </file>
@@ -176,7 +176,7 @@
     </font>
     <font>
       <b/>
-      <color rgb="FFC5221F"/>
+      <color rgb="FF137333"/>
       <sz val="10"/>
       <name val="Arial"/>
     </font>
@@ -195,7 +195,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFCE8E6"/>
+        <fgColor rgb="FFE6F4EA"/>
       </patternFill>
     </fill>
   </fills>
@@ -637,7 +637,7 @@
         <v>9</v>
       </c>
       <c r="B6" s="3">
-        <v>100</v>
+        <v>14550</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>